<commit_message>
chore(weekly-sync): auto-pull through 2026-06-28
</commit_message>
<xml_diff>
--- a/data/raw/returns/1p Returns.xlsx
+++ b/data/raw/returns/1p Returns.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Viewing Range=[23/03/26 - 20/06/26]  Currency=[INR]  View By=[ASIN]  Distributor View=[Manufacturing]  Source=[SP-API]</t>
+          <t>Viewing Range=[30/03/26 - 27/06/26]  Currency=[INR]  View By=[ASIN]  Distributor View=[Manufacturing]  Source=[SP-API]</t>
         </is>
       </c>
     </row>
@@ -493,10 +493,10 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>6030085.73</v>
+        <v>5977215.36</v>
       </c>
       <c r="F3" t="n">
-        <v>1478</v>
+        <v>1465</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -505,10 +505,10 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>1489</v>
+        <v>1467</v>
       </c>
       <c r="J3" t="n">
-        <v>352</v>
+        <v>362</v>
       </c>
     </row>
     <row r="4">
@@ -529,10 +529,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>5661283.31</v>
+        <v>5744261.53</v>
       </c>
       <c r="F4" t="n">
-        <v>2513</v>
+        <v>2548</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -541,10 +541,10 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>2518</v>
+        <v>2532</v>
       </c>
       <c r="J4" t="n">
-        <v>472</v>
+        <v>484</v>
       </c>
     </row>
     <row r="5">
@@ -565,10 +565,10 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2618449.45</v>
+        <v>2572028.31</v>
       </c>
       <c r="F5" t="n">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -577,10 +577,10 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="J5" t="n">
-        <v>102</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6">
@@ -601,10 +601,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2268633.87</v>
+        <v>2470895.85</v>
       </c>
       <c r="F6" t="n">
-        <v>381</v>
+        <v>412</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -613,10 +613,10 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>376</v>
+        <v>407</v>
       </c>
       <c r="J6" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7">
@@ -637,10 +637,10 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>2023673.8</v>
+        <v>2154327.23</v>
       </c>
       <c r="F7" t="n">
-        <v>466</v>
+        <v>495</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -649,10 +649,10 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>457</v>
+        <v>486</v>
       </c>
       <c r="J7" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8">
@@ -673,10 +673,10 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1519294.43</v>
+        <v>1521537.52</v>
       </c>
       <c r="F8" t="n">
-        <v>895</v>
+        <v>898</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -685,10 +685,10 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>892</v>
+        <v>899</v>
       </c>
       <c r="J8" t="n">
-        <v>161</v>
+        <v>171</v>
       </c>
     </row>
     <row r="9">
@@ -709,28 +709,28 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>1385000.81</v>
+        <v>1392965.12</v>
       </c>
       <c r="F9" t="n">
+        <v>593</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
         <v>591</v>
       </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
-        <v>600</v>
-      </c>
       <c r="J9" t="n">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>B0D3M1B4Z8</t>
+          <t>B0CF5TCQKL</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -745,10 +745,10 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>938360.23</v>
+        <v>900742.99</v>
       </c>
       <c r="F10" t="n">
-        <v>319</v>
+        <v>284</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -757,16 +757,16 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>318</v>
+        <v>285</v>
       </c>
       <c r="J10" t="n">
-        <v>67</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>B0CF5TCQKL</t>
+          <t>B0D3M1B4Z8</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -781,10 +781,10 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>902182.76</v>
+        <v>871429.8100000001</v>
       </c>
       <c r="F11" t="n">
-        <v>285</v>
+        <v>297</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -793,10 +793,10 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>281</v>
+        <v>298</v>
       </c>
       <c r="J11" t="n">
-        <v>27</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12">
@@ -829,7 +829,7 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="J12" t="n">
         <v>28</v>
@@ -853,10 +853,10 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>624458.4500000001</v>
+        <v>654878.78</v>
       </c>
       <c r="F13" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -865,10 +865,10 @@
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="J13" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14">
@@ -889,10 +889,10 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>591296.61</v>
+        <v>608244.09</v>
       </c>
       <c r="F14" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
@@ -901,10 +901,10 @@
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="J14" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15">
@@ -925,10 +925,10 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>546822.1</v>
+        <v>577651.5</v>
       </c>
       <c r="F15" t="n">
-        <v>408</v>
+        <v>429</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -937,16 +937,16 @@
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>408</v>
+        <v>429</v>
       </c>
       <c r="J15" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>B0B4G19R58</t>
+          <t>B0BPLWW72Y</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -961,10 +961,10 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>519244.17</v>
+        <v>545822.67</v>
       </c>
       <c r="F16" t="n">
-        <v>162</v>
+        <v>402</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -973,10 +973,10 @@
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>165</v>
+        <v>398</v>
       </c>
       <c r="J16" t="n">
-        <v>26</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17">
@@ -997,10 +997,10 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>498079.72</v>
+        <v>489015.31</v>
       </c>
       <c r="F17" t="n">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -1009,16 +1009,16 @@
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="J17" t="n">
-        <v>59</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>B0BPLWW72Y</t>
+          <t>B0B4G19R58</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -1033,10 +1033,10 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>473999.55</v>
+        <v>483829.77</v>
       </c>
       <c r="F18" t="n">
-        <v>353</v>
+        <v>151</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -1045,10 +1045,10 @@
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>351</v>
+        <v>147</v>
       </c>
       <c r="J18" t="n">
-        <v>49</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19">
@@ -1069,10 +1069,10 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>432957.34</v>
+        <v>428776.86</v>
       </c>
       <c r="F19" t="n">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -1081,16 +1081,16 @@
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="J19" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>B0B4KC7VBM</t>
+          <t>B0G53M9258</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -1105,10 +1105,10 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>393053.04</v>
+        <v>427391.64</v>
       </c>
       <c r="F20" t="n">
-        <v>201</v>
+        <v>78</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -1117,16 +1117,16 @@
         <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>201</v>
+        <v>76</v>
       </c>
       <c r="J20" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>B0G53M9258</t>
+          <t>B0B4KC7VBM</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -1141,10 +1141,10 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>366807.75</v>
+        <v>388055.57</v>
       </c>
       <c r="F21" t="n">
-        <v>67</v>
+        <v>198</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -1153,16 +1153,16 @@
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>66</v>
+        <v>198</v>
       </c>
       <c r="J21" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>B0CM6NVLT9</t>
+          <t>B0DT6T6N6B</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -1177,10 +1177,10 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>342405.7</v>
+        <v>338264.3</v>
       </c>
       <c r="F22" t="n">
-        <v>259</v>
+        <v>709</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -1189,10 +1189,10 @@
         <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>257</v>
+        <v>707</v>
       </c>
       <c r="J22" t="n">
-        <v>70</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23">
@@ -1213,10 +1213,10 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>339696.37</v>
+        <v>337409.94</v>
       </c>
       <c r="F23" t="n">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
@@ -1225,16 +1225,16 @@
         <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J23" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>B0DT6T6N6B</t>
+          <t>B0CM6NVLT9</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>334453.09</v>
+        <v>333504.85</v>
       </c>
       <c r="F24" t="n">
-        <v>706</v>
+        <v>252</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -1261,10 +1261,10 @@
         <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>711</v>
+        <v>255</v>
       </c>
       <c r="J24" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="25">
@@ -1285,10 +1285,10 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>235604.96</v>
+        <v>255175.28</v>
       </c>
       <c r="F25" t="n">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
@@ -1297,16 +1297,16 @@
         <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="J25" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>B0CM9HYVDM</t>
+          <t>B0BLJVJ2GN</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -1321,10 +1321,10 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>232254.96</v>
+        <v>239845.73</v>
       </c>
       <c r="F26" t="n">
-        <v>232</v>
+        <v>432</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
@@ -1333,10 +1333,10 @@
         <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>233</v>
+        <v>430</v>
       </c>
       <c r="J26" t="n">
-        <v>38</v>
+        <v>71</v>
       </c>
     </row>
     <row r="27">
@@ -1357,10 +1357,10 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>228191.18</v>
+        <v>236897.39</v>
       </c>
       <c r="F27" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
@@ -1369,10 +1369,10 @@
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="J27" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="28">
@@ -1393,10 +1393,10 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>227097.54</v>
+        <v>228961.1</v>
       </c>
       <c r="F28" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -1405,16 +1405,16 @@
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="J28" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>B0BLJVJ2GN</t>
+          <t>B0CM9HYVDM</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -1429,10 +1429,10 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>223895.73</v>
+        <v>225201.53</v>
       </c>
       <c r="F29" t="n">
-        <v>403</v>
+        <v>225</v>
       </c>
       <c r="G29" t="n">
         <v>0</v>
@@ -1441,16 +1441,16 @@
         <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>400</v>
+        <v>224</v>
       </c>
       <c r="J29" t="n">
-        <v>62</v>
+        <v>40</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>B0FQBX8J17</t>
+          <t>B0B4JRQP22</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1465,10 +1465,10 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>220101.48</v>
+        <v>214822.32</v>
       </c>
       <c r="F30" t="n">
-        <v>204</v>
+        <v>102</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
@@ -1477,16 +1477,16 @@
         <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>205</v>
+        <v>99</v>
       </c>
       <c r="J30" t="n">
-        <v>44</v>
+        <v>11</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>B0B4JRQP22</t>
+          <t>B0FQBX8J17</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1501,10 +1501,10 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>208468.92</v>
+        <v>212015.07</v>
       </c>
       <c r="F31" t="n">
-        <v>99</v>
+        <v>194</v>
       </c>
       <c r="G31" t="n">
         <v>0</v>
@@ -1513,16 +1513,16 @@
         <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>99</v>
+        <v>195</v>
       </c>
       <c r="J31" t="n">
-        <v>10</v>
+        <v>38</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>B0B4K87PR4</t>
+          <t>B0GN2LHJY4</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -1537,10 +1537,10 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>190907.63</v>
+        <v>206333.91</v>
       </c>
       <c r="F32" t="n">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="G32" t="n">
         <v>0</v>
@@ -1549,16 +1549,16 @@
         <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="J32" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>B0BPM2T7BQ</t>
+          <t>B0B4K87PR4</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -1573,10 +1573,10 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>189106.13</v>
+        <v>201643.96</v>
       </c>
       <c r="F33" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
@@ -1585,16 +1585,16 @@
         <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J33" t="n">
-        <v>23</v>
+        <v>5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>B0CM9KJZWQ</t>
+          <t>B0BPM2T7BQ</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -1609,10 +1609,10 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>178543.11</v>
+        <v>192749.33</v>
       </c>
       <c r="F34" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
@@ -1621,10 +1621,10 @@
         <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="J34" t="n">
-        <v>9</v>
+        <v>26</v>
       </c>
     </row>
     <row r="35">
@@ -1645,10 +1645,10 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>177760.99</v>
+        <v>190470.31</v>
       </c>
       <c r="F35" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -1657,16 +1657,16 @@
         <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="J35" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>B0GN2LHJY4</t>
+          <t>B0FQBTRM28</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -1681,10 +1681,10 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>175828.82</v>
+        <v>168818.66</v>
       </c>
       <c r="F36" t="n">
-        <v>22</v>
+        <v>100</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
@@ -1693,10 +1693,10 @@
         <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>22</v>
+        <v>99</v>
       </c>
       <c r="J36" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37">
@@ -1717,10 +1717,10 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>172683.86</v>
+        <v>166837.25</v>
       </c>
       <c r="F37" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
@@ -1729,22 +1729,22 @@
         <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="J37" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>B0DN6MNS1X</t>
+          <t>B07GVGMW59</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Audio Array</t>
+          <t>Tonor</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1753,10 +1753,10 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>167702.67</v>
+        <v>162989.71</v>
       </c>
       <c r="F38" t="n">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
@@ -1765,16 +1765,16 @@
         <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>41</v>
+        <v>71</v>
       </c>
       <c r="J38" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>B0DFMNGFTD</t>
+          <t>B0B4G7VWXD</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
@@ -1789,34 +1789,34 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>164294.13</v>
+        <v>158397.64</v>
       </c>
       <c r="F39" t="n">
+        <v>111</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" t="n">
+        <v>110</v>
+      </c>
+      <c r="J39" t="n">
         <v>31</v>
-      </c>
-      <c r="G39" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" t="n">
-        <v>31</v>
-      </c>
-      <c r="J39" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>B0FQBTRM28</t>
+          <t>B0CCV74CL7</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Audio Array</t>
+          <t>Tonor</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1825,10 +1825,10 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>161704.25</v>
+        <v>155962.72</v>
       </c>
       <c r="F40" t="n">
-        <v>96</v>
+        <v>64</v>
       </c>
       <c r="G40" t="n">
         <v>0</v>
@@ -1837,16 +1837,16 @@
         <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>97</v>
+        <v>64</v>
       </c>
       <c r="J40" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>B0CM6WH4ZT</t>
+          <t>B0CM9KJZWQ</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
@@ -1861,10 +1861,10 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>151356.73</v>
+        <v>154649.91</v>
       </c>
       <c r="F41" t="n">
-        <v>128</v>
+        <v>39</v>
       </c>
       <c r="G41" t="n">
         <v>0</v>
@@ -1873,22 +1873,22 @@
         <v>0</v>
       </c>
       <c r="I41" t="n">
-        <v>129</v>
+        <v>39</v>
       </c>
       <c r="J41" t="n">
-        <v>58</v>
+        <v>7</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>B0CCV74CL7</t>
+          <t>B0DFMNGFTD</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Tonor</t>
+          <t>Audio Array</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1897,10 +1897,10 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>151303.39</v>
+        <v>153956.86</v>
       </c>
       <c r="F42" t="n">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="G42" t="n">
         <v>0</v>
@@ -1909,7 +1909,7 @@
         <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="J42" t="n">
         <v>13</v>
@@ -1933,10 +1933,10 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>149591.65</v>
+        <v>150522.14</v>
       </c>
       <c r="F43" t="n">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="G43" t="n">
         <v>0</v>
@@ -1945,16 +1945,16 @@
         <v>0</v>
       </c>
       <c r="I43" t="n">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="J43" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>B0B4G7VWXD</t>
+          <t>B0DN6MNS1X</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -1969,10 +1969,10 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>148318.77</v>
+        <v>149749.83</v>
       </c>
       <c r="F44" t="n">
-        <v>104</v>
+        <v>36</v>
       </c>
       <c r="G44" t="n">
         <v>0</v>
@@ -1981,10 +1981,10 @@
         <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>105</v>
+        <v>36</v>
       </c>
       <c r="J44" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
     </row>
     <row r="45">
@@ -2005,10 +2005,10 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>146502.56</v>
+        <v>149637.3</v>
       </c>
       <c r="F45" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G45" t="n">
         <v>0</v>
@@ -2017,7 +2017,7 @@
         <v>0</v>
       </c>
       <c r="I45" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J45" t="n">
         <v>3</v>
@@ -2026,13 +2026,13 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>B0CQX3VB1R</t>
+          <t>B0FFB6YJM1</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Tonor</t>
+          <t>Audio Array</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2041,10 +2041,10 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>145156.67</v>
+        <v>147046.11</v>
       </c>
       <c r="F46" t="n">
-        <v>85</v>
+        <v>143</v>
       </c>
       <c r="G46" t="n">
         <v>0</v>
@@ -2053,22 +2053,22 @@
         <v>0</v>
       </c>
       <c r="I46" t="n">
-        <v>87</v>
+        <v>137</v>
       </c>
       <c r="J46" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>B07GVGMW59</t>
+          <t>B0G53KWRVW</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Tonor</t>
+          <t>Audio Array</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2077,10 +2077,10 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>142404.15</v>
+        <v>142739</v>
       </c>
       <c r="F47" t="n">
-        <v>63</v>
+        <v>16</v>
       </c>
       <c r="G47" t="n">
         <v>0</v>
@@ -2089,16 +2089,16 @@
         <v>0</v>
       </c>
       <c r="I47" t="n">
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="J47" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>B0FN7B3KWS</t>
+          <t>B0CM6WH4ZT</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
@@ -2113,10 +2113,10 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>132107.61</v>
+        <v>139500.79</v>
       </c>
       <c r="F48" t="n">
-        <v>13</v>
+        <v>118</v>
       </c>
       <c r="G48" t="n">
         <v>0</v>
@@ -2125,16 +2125,16 @@
         <v>0</v>
       </c>
       <c r="I48" t="n">
-        <v>13</v>
+        <v>118</v>
       </c>
       <c r="J48" t="n">
-        <v>3</v>
+        <v>62</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>B0D3M86SH1</t>
+          <t>B0FN7B3KWS</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
@@ -2149,10 +2149,10 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>130115.24</v>
+        <v>132107.61</v>
       </c>
       <c r="F49" t="n">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="G49" t="n">
         <v>0</v>
@@ -2161,16 +2161,16 @@
         <v>0</v>
       </c>
       <c r="I49" t="n">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="J49" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>B07WLWN2ZT</t>
+          <t>B01ISNU3X4</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -2185,10 +2185,10 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>119612.69</v>
+        <v>129073.32</v>
       </c>
       <c r="F50" t="n">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
@@ -2197,22 +2197,22 @@
         <v>0</v>
       </c>
       <c r="I50" t="n">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="J50" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>B0FFB6YJM1</t>
+          <t>B07WLWN2ZT</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Audio Array</t>
+          <t>Tonor</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>118677.44</v>
+        <v>128083.01</v>
       </c>
       <c r="F51" t="n">
-        <v>116</v>
+        <v>74</v>
       </c>
       <c r="G51" t="n">
         <v>0</v>
@@ -2233,16 +2233,16 @@
         <v>0</v>
       </c>
       <c r="I51" t="n">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="J51" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>B01ISNU3X4</t>
+          <t>B0CQX3VB1R</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
@@ -2257,10 +2257,10 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>117680.97</v>
+        <v>127369.42</v>
       </c>
       <c r="F52" t="n">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="G52" t="n">
         <v>0</v>
@@ -2269,22 +2269,22 @@
         <v>0</v>
       </c>
       <c r="I52" t="n">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="J52" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>B0B4G763WS</t>
+          <t>B08NDB5NWP</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Audio Array</t>
+          <t>Tonor</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2293,10 +2293,10 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>110546.69</v>
+        <v>126822.13</v>
       </c>
       <c r="F53" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="G53" t="n">
         <v>0</v>
@@ -2305,22 +2305,22 @@
         <v>0</v>
       </c>
       <c r="I53" t="n">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="J53" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>B08NDB5NWP</t>
+          <t>B0D3M86SH1</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Tonor</t>
+          <t>Audio Array</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2329,10 +2329,10 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>109031.44</v>
+        <v>125894.04</v>
       </c>
       <c r="F54" t="n">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="G54" t="n">
         <v>0</v>
@@ -2341,16 +2341,16 @@
         <v>0</v>
       </c>
       <c r="I54" t="n">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="J54" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>B0G3B677Z5</t>
+          <t>B0B4G763WS</t>
         </is>
       </c>
       <c r="B55" t="inlineStr"/>
@@ -2365,10 +2365,10 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>108172.88</v>
+        <v>120713.63</v>
       </c>
       <c r="F55" t="n">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="G55" t="n">
         <v>0</v>
@@ -2377,16 +2377,16 @@
         <v>0</v>
       </c>
       <c r="I55" t="n">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="J55" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>B0G53KWRVW</t>
+          <t>B0G39ZHDYP</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
@@ -2401,10 +2401,10 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>107149.16</v>
+        <v>119641.32</v>
       </c>
       <c r="F56" t="n">
-        <v>12</v>
+        <v>118</v>
       </c>
       <c r="G56" t="n">
         <v>0</v>
@@ -2413,16 +2413,16 @@
         <v>0</v>
       </c>
       <c r="I56" t="n">
-        <v>11</v>
+        <v>118</v>
       </c>
       <c r="J56" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>B0FQBWV1ST</t>
+          <t>B0D3LZWTHV</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
@@ -2437,10 +2437,10 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>102405.84</v>
+        <v>104830.47</v>
       </c>
       <c r="F57" t="n">
-        <v>61</v>
+        <v>36</v>
       </c>
       <c r="G57" t="n">
         <v>0</v>
@@ -2449,16 +2449,16 @@
         <v>0</v>
       </c>
       <c r="I57" t="n">
-        <v>61</v>
+        <v>36</v>
       </c>
       <c r="J57" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>B0D3LZWTHV</t>
+          <t>B0FQBWV1ST</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
@@ -2473,10 +2473,10 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>99069.45</v>
+        <v>100838.9</v>
       </c>
       <c r="F58" t="n">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="G58" t="n">
         <v>0</v>
@@ -2485,16 +2485,16 @@
         <v>0</v>
       </c>
       <c r="I58" t="n">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="J58" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>B0CBCB82MT</t>
+          <t>B0G3B677Z5</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
@@ -2509,10 +2509,10 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>98762.72</v>
+        <v>98427.96000000001</v>
       </c>
       <c r="F59" t="n">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="G59" t="n">
         <v>0</v>
@@ -2521,16 +2521,16 @@
         <v>0</v>
       </c>
       <c r="I59" t="n">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="J59" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>B0G39ZHDYP</t>
+          <t>B0FJ2JJZL3</t>
         </is>
       </c>
       <c r="B60" t="inlineStr"/>
@@ -2545,10 +2545,10 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>98303.22</v>
+        <v>98299.98000000001</v>
       </c>
       <c r="F60" t="n">
-        <v>97</v>
+        <v>6</v>
       </c>
       <c r="G60" t="n">
         <v>0</v>
@@ -2557,16 +2557,16 @@
         <v>0</v>
       </c>
       <c r="I60" t="n">
-        <v>95</v>
+        <v>6</v>
       </c>
       <c r="J60" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>B0FJ2JJZL3</t>
+          <t>B0B4G1HPL5</t>
         </is>
       </c>
       <c r="B61" t="inlineStr"/>
@@ -2581,10 +2581,10 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>98299.98000000001</v>
+        <v>95316.03999999999</v>
       </c>
       <c r="F61" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="G61" t="n">
         <v>0</v>
@@ -2593,16 +2593,16 @@
         <v>0</v>
       </c>
       <c r="I61" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="J61" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>B0B4G1HPL5</t>
+          <t>B0CBCB82MT</t>
         </is>
       </c>
       <c r="B62" t="inlineStr"/>
@@ -2617,10 +2617,10 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>91333.84</v>
+        <v>89637.25999999999</v>
       </c>
       <c r="F62" t="n">
-        <v>23</v>
+        <v>64</v>
       </c>
       <c r="G62" t="n">
         <v>0</v>
@@ -2629,16 +2629,16 @@
         <v>0</v>
       </c>
       <c r="I62" t="n">
+        <v>65</v>
+      </c>
+      <c r="J62" t="n">
         <v>24</v>
-      </c>
-      <c r="J62" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>B0BQ7H7418</t>
+          <t>B0FTVVLNS9</t>
         </is>
       </c>
       <c r="B63" t="inlineStr"/>
@@ -2653,10 +2653,10 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>87389.8</v>
+        <v>89483.89999999999</v>
       </c>
       <c r="F63" t="n">
-        <v>80</v>
+        <v>9</v>
       </c>
       <c r="G63" t="n">
         <v>0</v>
@@ -2665,16 +2665,16 @@
         <v>0</v>
       </c>
       <c r="I63" t="n">
-        <v>80</v>
+        <v>9</v>
       </c>
       <c r="J63" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>B0B4G8ZB64</t>
+          <t>B0BQ7H7418</t>
         </is>
       </c>
       <c r="B64" t="inlineStr"/>
@@ -2689,10 +2689,10 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>83450.03</v>
+        <v>88490.64999999999</v>
       </c>
       <c r="F64" t="n">
-        <v>106</v>
+        <v>81</v>
       </c>
       <c r="G64" t="n">
         <v>0</v>
@@ -2701,16 +2701,16 @@
         <v>0</v>
       </c>
       <c r="I64" t="n">
-        <v>109</v>
+        <v>80</v>
       </c>
       <c r="J64" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>B0GKPXQ8G3</t>
+          <t>B0B4G8ZB64</t>
         </is>
       </c>
       <c r="B65" t="inlineStr"/>
@@ -2725,10 +2725,10 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>80756.64</v>
+        <v>82857.68000000001</v>
       </c>
       <c r="F65" t="n">
-        <v>28</v>
+        <v>105</v>
       </c>
       <c r="G65" t="n">
         <v>0</v>
@@ -2737,10 +2737,10 @@
         <v>0</v>
       </c>
       <c r="I65" t="n">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="J65" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="66">
@@ -2761,10 +2761,10 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>79550.75999999999</v>
+        <v>82219.39999999999</v>
       </c>
       <c r="F66" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G66" t="n">
         <v>0</v>
@@ -2773,16 +2773,16 @@
         <v>0</v>
       </c>
       <c r="I66" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J66" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>B0FTVVLNS9</t>
+          <t>B0GKPXQ8G3</t>
         </is>
       </c>
       <c r="B67" t="inlineStr"/>
@@ -2797,10 +2797,10 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>79400</v>
+        <v>80315.26000000001</v>
       </c>
       <c r="F67" t="n">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="G67" t="n">
         <v>0</v>
@@ -2809,16 +2809,16 @@
         <v>0</v>
       </c>
       <c r="I67" t="n">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="J67" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>B0FF9R3GKK</t>
+          <t>B0DFMLXD9S</t>
         </is>
       </c>
       <c r="B68" t="inlineStr"/>
@@ -2833,10 +2833,10 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>78111.85000000001</v>
+        <v>76937.06</v>
       </c>
       <c r="F68" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="G68" t="n">
         <v>0</v>
@@ -2845,16 +2845,16 @@
         <v>0</v>
       </c>
       <c r="I68" t="n">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="J68" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>B0DFMKY4TT</t>
+          <t>B0FTVV1QJY</t>
         </is>
       </c>
       <c r="B69" t="inlineStr"/>
@@ -2869,10 +2869,10 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>75277.91</v>
+        <v>75880.59</v>
       </c>
       <c r="F69" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="G69" t="n">
         <v>0</v>
@@ -2881,16 +2881,16 @@
         <v>0</v>
       </c>
       <c r="I69" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="J69" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>B0DFMLXD9S</t>
+          <t>B0GN8RQJRG</t>
         </is>
       </c>
       <c r="B70" t="inlineStr"/>
@@ -2905,10 +2905,10 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>73209.18000000001</v>
+        <v>73921.96000000001</v>
       </c>
       <c r="F70" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G70" t="n">
         <v>0</v>
@@ -2917,16 +2917,16 @@
         <v>0</v>
       </c>
       <c r="I70" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="J70" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>B0FTVV1QJY</t>
+          <t>B0DN6PFWNK</t>
         </is>
       </c>
       <c r="B71" t="inlineStr"/>
@@ -2941,10 +2941,10 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>71813.64</v>
+        <v>73883.89999999999</v>
       </c>
       <c r="F71" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G71" t="n">
         <v>0</v>
@@ -2953,22 +2953,22 @@
         <v>0</v>
       </c>
       <c r="I71" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J71" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>B0GN8RQJRG</t>
+          <t>B0CQX4K9P5</t>
         </is>
       </c>
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Audio Array</t>
+          <t>Tonor</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2977,10 +2977,10 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>70532.98</v>
+        <v>71049.12</v>
       </c>
       <c r="F72" t="n">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="G72" t="n">
         <v>0</v>
@@ -2989,10 +2989,10 @@
         <v>0</v>
       </c>
       <c r="I72" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="J72" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73">
@@ -3013,7 +3013,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>67978.55</v>
+        <v>67893.81</v>
       </c>
       <c r="F73" t="n">
         <v>28</v>
@@ -3025,22 +3025,22 @@
         <v>0</v>
       </c>
       <c r="I73" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J73" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>B0FPR962YS</t>
+          <t>B078WNW4YW</t>
         </is>
       </c>
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Audio Array</t>
+          <t>Tonor</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -3049,10 +3049,10 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>67847.98</v>
+        <v>67777.89999999999</v>
       </c>
       <c r="F74" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="G74" t="n">
         <v>0</v>
@@ -3061,22 +3061,22 @@
         <v>0</v>
       </c>
       <c r="I74" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="J74" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>B078WNW4YW</t>
+          <t>B0DFMKY4TT</t>
         </is>
       </c>
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Tonor</t>
+          <t>Audio Array</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -3085,10 +3085,10 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>67777.89999999999</v>
+        <v>66127.91</v>
       </c>
       <c r="F75" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="G75" t="n">
         <v>0</v>
@@ -3097,16 +3097,16 @@
         <v>0</v>
       </c>
       <c r="I75" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="J75" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>B0B4G8PH2P</t>
+          <t>B0FF9R3GKK</t>
         </is>
       </c>
       <c r="B76" t="inlineStr"/>
@@ -3121,10 +3121,10 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>65223.71</v>
+        <v>65827.95</v>
       </c>
       <c r="F76" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="G76" t="n">
         <v>0</v>
@@ -3133,16 +3133,16 @@
         <v>0</v>
       </c>
       <c r="I76" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="J76" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>B0DN6PFWNK</t>
+          <t>B0B4G8PH2P</t>
         </is>
       </c>
       <c r="B77" t="inlineStr"/>
@@ -3157,10 +3157,10 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>65072.03</v>
+        <v>65223.7</v>
       </c>
       <c r="F77" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="G77" t="n">
         <v>0</v>
@@ -3169,16 +3169,16 @@
         <v>0</v>
       </c>
       <c r="I77" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="J77" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>B0CBC7QMNV</t>
+          <t>B0FPR962YS</t>
         </is>
       </c>
       <c r="B78" t="inlineStr"/>
@@ -3193,10 +3193,10 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>61593.19</v>
+        <v>64840.36</v>
       </c>
       <c r="F78" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G78" t="n">
         <v>0</v>
@@ -3205,16 +3205,16 @@
         <v>0</v>
       </c>
       <c r="I78" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="J78" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>B0FJ2DT13L</t>
+          <t>B0GXPBHDRF</t>
         </is>
       </c>
       <c r="B79" t="inlineStr"/>
@@ -3229,10 +3229,10 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>55451.64</v>
+        <v>61516.64999999999</v>
       </c>
       <c r="F79" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G79" t="n">
         <v>0</v>
@@ -3241,16 +3241,16 @@
         <v>0</v>
       </c>
       <c r="I79" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="J79" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>B0B4G94VP3</t>
+          <t>B0G53KWRWH</t>
         </is>
       </c>
       <c r="B80" t="inlineStr"/>
@@ -3265,10 +3265,10 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>54804.05</v>
+        <v>58472.04</v>
       </c>
       <c r="F80" t="n">
-        <v>131</v>
+        <v>3</v>
       </c>
       <c r="G80" t="n">
         <v>0</v>
@@ -3277,22 +3277,22 @@
         <v>0</v>
       </c>
       <c r="I80" t="n">
-        <v>134</v>
+        <v>3</v>
       </c>
       <c r="J80" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>B0BTCXQQ6M</t>
+          <t>B0G3B152FR</t>
         </is>
       </c>
       <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Tonor</t>
+          <t>Audio Array</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3301,10 +3301,10 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>54770.41</v>
+        <v>57766.04</v>
       </c>
       <c r="F81" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="G81" t="n">
         <v>0</v>
@@ -3313,7 +3313,7 @@
         <v>0</v>
       </c>
       <c r="I81" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="J81" t="n">
         <v>4</v>
@@ -3322,13 +3322,13 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>B0FJ8PZ9H7</t>
+          <t>B0BTCXQQ6M</t>
         </is>
       </c>
       <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Audio Array</t>
+          <t>Tonor</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3337,10 +3337,10 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>54327.64</v>
+        <v>54770.41</v>
       </c>
       <c r="F82" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="G82" t="n">
         <v>0</v>
@@ -3349,16 +3349,16 @@
         <v>0</v>
       </c>
       <c r="I82" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="J82" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>B0CH4T2BJD</t>
+          <t>B0B4G94VP3</t>
         </is>
       </c>
       <c r="B83" t="inlineStr"/>
@@ -3373,10 +3373,10 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>53474.08</v>
+        <v>53535.41</v>
       </c>
       <c r="F83" t="n">
-        <v>27</v>
+        <v>128</v>
       </c>
       <c r="G83" t="n">
         <v>0</v>
@@ -3385,16 +3385,16 @@
         <v>0</v>
       </c>
       <c r="I83" t="n">
-        <v>28</v>
+        <v>127</v>
       </c>
       <c r="J83" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>B0B4G1PXWV</t>
+          <t>B0FJ2DT13L</t>
         </is>
       </c>
       <c r="B84" t="inlineStr"/>
@@ -3409,10 +3409,10 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>53436.39999999999</v>
+        <v>52105.02</v>
       </c>
       <c r="F84" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="G84" t="n">
         <v>0</v>
@@ -3421,16 +3421,16 @@
         <v>0</v>
       </c>
       <c r="I84" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="J84" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>B0G3B152FR</t>
+          <t>B0DFMLS8JG</t>
         </is>
       </c>
       <c r="B85" t="inlineStr"/>
@@ -3445,10 +3445,10 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>52938.08</v>
+        <v>50833.9</v>
       </c>
       <c r="F85" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="G85" t="n">
         <v>0</v>
@@ -3457,22 +3457,22 @@
         <v>0</v>
       </c>
       <c r="I85" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="J85" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>B0CQX4K9P5</t>
+          <t>B0CH4T2BJD</t>
         </is>
       </c>
       <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Tonor</t>
+          <t>Audio Array</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -3481,10 +3481,10 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>50720.33</v>
+        <v>49639.88</v>
       </c>
       <c r="F86" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G86" t="n">
         <v>0</v>
@@ -3493,22 +3493,22 @@
         <v>0</v>
       </c>
       <c r="I86" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="J86" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>B0BRKFP94K</t>
+          <t>B0CBC7QMNV</t>
         </is>
       </c>
       <c r="B87" t="inlineStr"/>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Tonor</t>
+          <t>Audio Array</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -3517,10 +3517,10 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>50264.36</v>
+        <v>49223.71</v>
       </c>
       <c r="F87" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G87" t="n">
         <v>0</v>
@@ -3529,16 +3529,16 @@
         <v>0</v>
       </c>
       <c r="I87" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J87" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>B0DFMLS8JG</t>
+          <t>B0B4G1PXWV</t>
         </is>
       </c>
       <c r="B88" t="inlineStr"/>
@@ -3553,10 +3553,10 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>47444.92</v>
+        <v>48777.94</v>
       </c>
       <c r="F88" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="G88" t="n">
         <v>0</v>
@@ -3565,10 +3565,10 @@
         <v>0</v>
       </c>
       <c r="I88" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="J88" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="89">
@@ -3604,13 +3604,13 @@
         <v>8</v>
       </c>
       <c r="J89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>B0FJ8S5XJ8</t>
+          <t>B0CM9P5CCK</t>
         </is>
       </c>
       <c r="B90" t="inlineStr"/>
@@ -3625,10 +3625,10 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>45081.36</v>
+        <v>45960.23</v>
       </c>
       <c r="F90" t="n">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="G90" t="n">
         <v>0</v>
@@ -3637,16 +3637,16 @@
         <v>0</v>
       </c>
       <c r="I90" t="n">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="J90" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>B0G3Q59X8C</t>
+          <t>B0CH4PMR8K</t>
         </is>
       </c>
       <c r="B91" t="inlineStr"/>
@@ -3661,10 +3661,10 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>43451.64</v>
+        <v>45818.50999999999</v>
       </c>
       <c r="F91" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="G91" t="n">
         <v>0</v>
@@ -3673,16 +3673,16 @@
         <v>0</v>
       </c>
       <c r="I91" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="J91" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>B0D3Q2T5XX</t>
+          <t>B0FJ8S5XJ8</t>
         </is>
       </c>
       <c r="B92" t="inlineStr"/>
@@ -3697,10 +3697,10 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>41940.71999999999</v>
+        <v>45081.36</v>
       </c>
       <c r="F92" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G92" t="n">
         <v>0</v>
@@ -3709,7 +3709,7 @@
         <v>0</v>
       </c>
       <c r="I92" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="J92" t="n">
         <v>1</v>
@@ -3718,7 +3718,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>B0CM9P5CCK</t>
+          <t>B0FJ2K95XT</t>
         </is>
       </c>
       <c r="B93" t="inlineStr"/>
@@ -3733,10 +3733,10 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>41640.73</v>
+        <v>41178.78</v>
       </c>
       <c r="F93" t="n">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="G93" t="n">
         <v>0</v>
@@ -3745,16 +3745,16 @@
         <v>0</v>
       </c>
       <c r="I93" t="n">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="J93" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>B0G53KWRWH</t>
+          <t>B0GN8MMKY1</t>
         </is>
       </c>
       <c r="B94" t="inlineStr"/>
@@ -3769,10 +3769,10 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>38981.36</v>
+        <v>40498.27</v>
       </c>
       <c r="F94" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="G94" t="n">
         <v>0</v>
@@ -3781,16 +3781,16 @@
         <v>0</v>
       </c>
       <c r="I94" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="J94" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>B0GXPBHDRF</t>
+          <t>B0CF5RRTDJ</t>
         </is>
       </c>
       <c r="B95" t="inlineStr"/>
@@ -3805,34 +3805,34 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>37791.21</v>
+        <v>35744.88</v>
       </c>
       <c r="F95" t="n">
+        <v>21</v>
+      </c>
+      <c r="G95" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" t="n">
+        <v>0</v>
+      </c>
+      <c r="I95" t="n">
+        <v>21</v>
+      </c>
+      <c r="J95" t="n">
         <v>6</v>
-      </c>
-      <c r="G95" t="n">
-        <v>0</v>
-      </c>
-      <c r="H95" t="n">
-        <v>0</v>
-      </c>
-      <c r="I95" t="n">
-        <v>6</v>
-      </c>
-      <c r="J95" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>B0DFMMTWLY</t>
+          <t>B082W4B7SX</t>
         </is>
       </c>
       <c r="B96" t="inlineStr"/>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Audio Array</t>
+          <t>Tonor</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -3841,10 +3841,10 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>37313.54</v>
+        <v>34985.56</v>
       </c>
       <c r="F96" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="G96" t="n">
         <v>0</v>
@@ -3853,16 +3853,16 @@
         <v>0</v>
       </c>
       <c r="I96" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="J96" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>B0FJ2K95XT</t>
+          <t>B0G3Q59X8C</t>
         </is>
       </c>
       <c r="B97" t="inlineStr"/>
@@ -3877,10 +3877,10 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>36603.36</v>
+        <v>34955.56</v>
       </c>
       <c r="F97" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="G97" t="n">
         <v>0</v>
@@ -3889,16 +3889,16 @@
         <v>0</v>
       </c>
       <c r="I97" t="n">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="J97" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>B0CH4PMR8K</t>
+          <t>B0CJR76Y7G</t>
         </is>
       </c>
       <c r="B98" t="inlineStr"/>
@@ -3913,10 +3913,10 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>36332.95</v>
+        <v>34323.77</v>
       </c>
       <c r="F98" t="n">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="G98" t="n">
         <v>0</v>
@@ -3925,16 +3925,16 @@
         <v>0</v>
       </c>
       <c r="I98" t="n">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="J98" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>B0GN8MMKY1</t>
+          <t>B0D3Q2T5XX</t>
         </is>
       </c>
       <c r="B99" t="inlineStr"/>
@@ -3949,10 +3949,10 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>33720.31</v>
+        <v>33467.84</v>
       </c>
       <c r="F99" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G99" t="n">
         <v>0</v>
@@ -3961,22 +3961,22 @@
         <v>0</v>
       </c>
       <c r="I99" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J99" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>B0B4G59Y8W</t>
+          <t>B0BRKFP94K</t>
         </is>
       </c>
       <c r="B100" t="inlineStr"/>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Audio Array</t>
+          <t>Tonor</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -3985,10 +3985,10 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>33111.86</v>
+        <v>33319.46</v>
       </c>
       <c r="F100" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G100" t="n">
         <v>0</v>
@@ -3997,16 +3997,16 @@
         <v>0</v>
       </c>
       <c r="I100" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="J100" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>B0CJR76Y7G</t>
+          <t>B0DFMMTWLY</t>
         </is>
       </c>
       <c r="B101" t="inlineStr"/>
@@ -4021,10 +4021,10 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>32884.8</v>
+        <v>32400.82</v>
       </c>
       <c r="F101" t="n">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="G101" t="n">
         <v>0</v>
@@ -4033,10 +4033,10 @@
         <v>0</v>
       </c>
       <c r="I101" t="n">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="J101" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="102">
@@ -4078,13 +4078,13 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>B082W4B7SX</t>
+          <t>B0FJ8PZ9H7</t>
         </is>
       </c>
       <c r="B103" t="inlineStr"/>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Tonor</t>
+          <t>Audio Array</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -4093,10 +4093,10 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>30834.72</v>
+        <v>31617.49</v>
       </c>
       <c r="F103" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="G103" t="n">
         <v>0</v>
@@ -4105,16 +4105,16 @@
         <v>0</v>
       </c>
       <c r="I103" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="J103" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>B0CM9L1QZG</t>
+          <t>B0B4G59Y8W</t>
         </is>
       </c>
       <c r="B104" t="inlineStr"/>
@@ -4129,10 +4129,10 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>27419.48</v>
+        <v>31248.3</v>
       </c>
       <c r="F104" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="G104" t="n">
         <v>0</v>
@@ -4141,16 +4141,16 @@
         <v>0</v>
       </c>
       <c r="I104" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="J104" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>B0CF5RRTDJ</t>
+          <t>B0FTVSH458</t>
         </is>
       </c>
       <c r="B105" t="inlineStr"/>
@@ -4165,10 +4165,10 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>27274.55</v>
+        <v>26058.22</v>
       </c>
       <c r="F105" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G105" t="n">
         <v>0</v>
@@ -4177,10 +4177,10 @@
         <v>0</v>
       </c>
       <c r="I105" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="J105" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="106">
@@ -4201,10 +4201,10 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>25630.25</v>
+        <v>24914.89</v>
       </c>
       <c r="F106" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G106" t="n">
         <v>0</v>
@@ -4213,16 +4213,16 @@
         <v>0</v>
       </c>
       <c r="I106" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="J106" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>B0DN6LJZBR</t>
+          <t>B0GXP97CZG</t>
         </is>
       </c>
       <c r="B107" t="inlineStr"/>
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>23892.37</v>
+        <v>24487.97</v>
       </c>
       <c r="F107" t="n">
         <v>7</v>
@@ -4252,13 +4252,13 @@
         <v>7</v>
       </c>
       <c r="J107" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>B0CH4R1V6S</t>
+          <t>B0DN6LJZBR</t>
         </is>
       </c>
       <c r="B108" t="inlineStr"/>
@@ -4273,10 +4273,10 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>23255.11</v>
+        <v>23892.37</v>
       </c>
       <c r="F108" t="n">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="G108" t="n">
         <v>0</v>
@@ -4285,22 +4285,22 @@
         <v>0</v>
       </c>
       <c r="I108" t="n">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="J108" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>B0CSCT63BL</t>
+          <t>B0CH4R1V6S</t>
         </is>
       </c>
       <c r="B109" t="inlineStr"/>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Tonor</t>
+          <t>Audio Array</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -4309,10 +4309,10 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>22829.65</v>
+        <v>22662.73</v>
       </c>
       <c r="F109" t="n">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="G109" t="n">
         <v>0</v>
@@ -4321,10 +4321,10 @@
         <v>0</v>
       </c>
       <c r="I109" t="n">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="J109" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
     </row>
     <row r="110">
@@ -4357,16 +4357,16 @@
         <v>0</v>
       </c>
       <c r="I110" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J110" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>B0FTVSH458</t>
+          <t>B0CM9L1QZG</t>
         </is>
       </c>
       <c r="B111" t="inlineStr"/>
@@ -4381,10 +4381,10 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>22115.85</v>
+        <v>20560.16</v>
       </c>
       <c r="F111" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="G111" t="n">
         <v>0</v>
@@ -4393,22 +4393,22 @@
         <v>0</v>
       </c>
       <c r="I111" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="J111" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>B0G53PRM34</t>
+          <t>B0CFKHCQ8W</t>
         </is>
       </c>
       <c r="B112" t="inlineStr"/>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Audio Array</t>
+          <t>Tonor</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -4417,10 +4417,10 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>21268.64</v>
+        <v>19905.91</v>
       </c>
       <c r="F112" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="G112" t="n">
         <v>0</v>
@@ -4429,16 +4429,16 @@
         <v>0</v>
       </c>
       <c r="I112" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J112" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>B0GXP97CZG</t>
+          <t>B0B4G89VQJ</t>
         </is>
       </c>
       <c r="B113" t="inlineStr"/>
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>21200.69</v>
+        <v>19825.44</v>
       </c>
       <c r="F113" t="n">
         <v>6</v>
@@ -4468,19 +4468,19 @@
         <v>6</v>
       </c>
       <c r="J113" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>B0CBCB9S14</t>
+          <t>B0CSCT63BL</t>
         </is>
       </c>
       <c r="B114" t="inlineStr"/>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Audio Array</t>
+          <t>Tonor</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -4489,10 +4489,10 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>21072.06</v>
+        <v>18594.05</v>
       </c>
       <c r="F114" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G114" t="n">
         <v>0</v>
@@ -4501,7 +4501,7 @@
         <v>0</v>
       </c>
       <c r="I114" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J114" t="n">
         <v>2</v>
@@ -4510,13 +4510,13 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>B0CFKHCQ8W</t>
+          <t>B0G53CB72D</t>
         </is>
       </c>
       <c r="B115" t="inlineStr"/>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Tonor</t>
+          <t>Audio Array</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -4525,10 +4525,10 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>19905.91</v>
+        <v>17795.76</v>
       </c>
       <c r="F115" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="G115" t="n">
         <v>0</v>
@@ -4537,22 +4537,22 @@
         <v>0</v>
       </c>
       <c r="I115" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="J115" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>B0B4G89VQJ</t>
+          <t>B0BBL47VR5</t>
         </is>
       </c>
       <c r="B116" t="inlineStr"/>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Audio Array</t>
+          <t>Tonor</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -4561,7 +4561,7 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>19825.44</v>
+        <v>17752.53</v>
       </c>
       <c r="F116" t="n">
         <v>6</v>
@@ -4582,13 +4582,13 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>B08V1JS3NY</t>
+          <t>B0CBCB9S14</t>
         </is>
       </c>
       <c r="B117" t="inlineStr"/>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Tonor</t>
+          <t>Audio Array</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -4597,10 +4597,10 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>19680.49</v>
+        <v>16836.46</v>
       </c>
       <c r="F117" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G117" t="n">
         <v>0</v>
@@ -4609,16 +4609,16 @@
         <v>0</v>
       </c>
       <c r="I117" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J117" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>B0G53CB72D</t>
+          <t>B0FJ2J6MTF</t>
         </is>
       </c>
       <c r="B118" t="inlineStr"/>
@@ -4633,10 +4633,10 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>17795.76</v>
+        <v>15690.68</v>
       </c>
       <c r="F118" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G118" t="n">
         <v>0</v>
@@ -4645,7 +4645,7 @@
         <v>0</v>
       </c>
       <c r="I118" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J118" t="n">
         <v>0</v>
@@ -4654,13 +4654,13 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>B0BBL47VR5</t>
+          <t>B0FJ2LQT7K</t>
         </is>
       </c>
       <c r="B119" t="inlineStr"/>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Tonor</t>
+          <t>Audio Array</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -4669,10 +4669,10 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>17752.53</v>
+        <v>15591.52</v>
       </c>
       <c r="F119" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G119" t="n">
         <v>0</v>
@@ -4681,10 +4681,10 @@
         <v>0</v>
       </c>
       <c r="I119" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J119" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="120">
@@ -4705,10 +4705,10 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>16942.4</v>
+        <v>14824.6</v>
       </c>
       <c r="F120" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G120" t="n">
         <v>0</v>
@@ -4717,7 +4717,7 @@
         <v>0</v>
       </c>
       <c r="I120" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J120" t="n">
         <v>2</v>
@@ -4726,13 +4726,13 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>B0FJ2J6MTF</t>
+          <t>B08V1JS3NY</t>
         </is>
       </c>
       <c r="B121" t="inlineStr"/>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Audio Array</t>
+          <t>Tonor</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -4741,28 +4741,28 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>15690.68</v>
+        <v>14088.97</v>
       </c>
       <c r="F121" t="n">
+        <v>5</v>
+      </c>
+      <c r="G121" t="n">
+        <v>0</v>
+      </c>
+      <c r="H121" t="n">
+        <v>0</v>
+      </c>
+      <c r="I121" t="n">
+        <v>5</v>
+      </c>
+      <c r="J121" t="n">
         <v>4</v>
-      </c>
-      <c r="G121" t="n">
-        <v>0</v>
-      </c>
-      <c r="H121" t="n">
-        <v>0</v>
-      </c>
-      <c r="I121" t="n">
-        <v>4</v>
-      </c>
-      <c r="J121" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>B0FJ2LQT7K</t>
+          <t>B0G53PRM34</t>
         </is>
       </c>
       <c r="B122" t="inlineStr"/>
@@ -4777,7 +4777,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>15591.52</v>
+        <v>14066.1</v>
       </c>
       <c r="F122" t="n">
         <v>2</v>
@@ -4792,19 +4792,19 @@
         <v>2</v>
       </c>
       <c r="J122" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>B0FPR7VFCH</t>
+          <t>B07TSN2H9D</t>
         </is>
       </c>
       <c r="B123" t="inlineStr"/>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Audio Array</t>
+          <t>Tonor</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -4813,10 +4813,10 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>15246.6</v>
+        <v>13894.91</v>
       </c>
       <c r="F123" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G123" t="n">
         <v>0</v>
@@ -4825,16 +4825,16 @@
         <v>0</v>
       </c>
       <c r="I123" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J123" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>B0FLYJFC22</t>
+          <t>B0C55MY66L</t>
         </is>
       </c>
       <c r="B124" t="inlineStr"/>
@@ -4849,10 +4849,10 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>13934.76</v>
+        <v>12160.18</v>
       </c>
       <c r="F124" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G124" t="n">
         <v>0</v>
@@ -4861,22 +4861,22 @@
         <v>0</v>
       </c>
       <c r="I124" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J124" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>B0FLYHJ6DK</t>
+          <t>B089FVQD3Z</t>
         </is>
       </c>
       <c r="B125" t="inlineStr"/>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Audio Array</t>
+          <t>Tonor</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -4885,10 +4885,10 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>13728.78</v>
+        <v>11860.15</v>
       </c>
       <c r="F125" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G125" t="n">
         <v>0</v>
@@ -4897,16 +4897,16 @@
         <v>0</v>
       </c>
       <c r="I125" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="J125" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>B0C55MY66L</t>
+          <t>B0FLYHJ6DK</t>
         </is>
       </c>
       <c r="B126" t="inlineStr"/>
@@ -4921,28 +4921,28 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>12160.18</v>
+        <v>10967.78</v>
       </c>
       <c r="F126" t="n">
+        <v>8</v>
+      </c>
+      <c r="G126" t="n">
+        <v>0</v>
+      </c>
+      <c r="H126" t="n">
+        <v>0</v>
+      </c>
+      <c r="I126" t="n">
+        <v>8</v>
+      </c>
+      <c r="J126" t="n">
         <v>4</v>
-      </c>
-      <c r="G126" t="n">
-        <v>0</v>
-      </c>
-      <c r="H126" t="n">
-        <v>0</v>
-      </c>
-      <c r="I126" t="n">
-        <v>4</v>
-      </c>
-      <c r="J126" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>B0BLKF46QG</t>
+          <t>B0FN7C25VS</t>
         </is>
       </c>
       <c r="B127" t="inlineStr"/>
@@ -4957,10 +4957,10 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>11407.62</v>
+        <v>10505.94</v>
       </c>
       <c r="F127" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G127" t="n">
         <v>0</v>
@@ -4969,16 +4969,16 @@
         <v>0</v>
       </c>
       <c r="I127" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="J127" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>B0FN7C25VS</t>
+          <t>B0FPR7VFCH</t>
         </is>
       </c>
       <c r="B128" t="inlineStr"/>
@@ -4993,28 +4993,28 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>10505.94</v>
+        <v>10164.4</v>
       </c>
       <c r="F128" t="n">
+        <v>6</v>
+      </c>
+      <c r="G128" t="n">
+        <v>0</v>
+      </c>
+      <c r="H128" t="n">
+        <v>0</v>
+      </c>
+      <c r="I128" t="n">
+        <v>6</v>
+      </c>
+      <c r="J128" t="n">
         <v>3</v>
-      </c>
-      <c r="G128" t="n">
-        <v>0</v>
-      </c>
-      <c r="H128" t="n">
-        <v>0</v>
-      </c>
-      <c r="I128" t="n">
-        <v>4</v>
-      </c>
-      <c r="J128" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>B0CH4RT4P8</t>
+          <t>B0FLYJFC22</t>
         </is>
       </c>
       <c r="B129" t="inlineStr"/>
@@ -5029,10 +5029,10 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>9835.77</v>
+        <v>9953.4</v>
       </c>
       <c r="F129" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G129" t="n">
         <v>0</v>
@@ -5041,22 +5041,22 @@
         <v>0</v>
       </c>
       <c r="I129" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J129" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>B089FVQD3Z</t>
+          <t>B0CH4RT4P8</t>
         </is>
       </c>
       <c r="B130" t="inlineStr"/>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Tonor</t>
+          <t>Audio Array</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="E130" t="n">
-        <v>9488.120000000001</v>
+        <v>9835.77</v>
       </c>
       <c r="F130" t="n">
         <v>4</v>
@@ -5077,16 +5077,16 @@
         <v>0</v>
       </c>
       <c r="I130" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J130" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>B0G53LZNY3</t>
+          <t>B0BLKF46QG</t>
         </is>
       </c>
       <c r="B131" t="inlineStr"/>
@@ -5101,10 +5101,10 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>9320.34</v>
+        <v>9121.18</v>
       </c>
       <c r="F131" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G131" t="n">
         <v>0</v>
@@ -5113,16 +5113,16 @@
         <v>0</v>
       </c>
       <c r="I131" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J131" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>B0FJ2HZCVN</t>
+          <t>B0GW96SHSK</t>
         </is>
       </c>
       <c r="B132" t="inlineStr"/>
@@ -5137,10 +5137,10 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>7626.27</v>
+        <v>8641.530000000001</v>
       </c>
       <c r="F132" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G132" t="n">
         <v>0</v>
@@ -5149,7 +5149,7 @@
         <v>0</v>
       </c>
       <c r="I132" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J132" t="n">
         <v>0</v>
@@ -5158,13 +5158,13 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>B07TSN2H9D</t>
+          <t>B0FJ2HZCVN</t>
         </is>
       </c>
       <c r="B133" t="inlineStr"/>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Tonor</t>
+          <t>Audio Array</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -5173,10 +5173,10 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>6947.45</v>
+        <v>7626.27</v>
       </c>
       <c r="F133" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G133" t="n">
         <v>0</v>
@@ -5185,7 +5185,7 @@
         <v>0</v>
       </c>
       <c r="I133" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J133" t="n">
         <v>0</v>
@@ -5194,13 +5194,13 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>B09Z5Q194D</t>
+          <t>B0FN7FYZM3</t>
         </is>
       </c>
       <c r="B134" t="inlineStr"/>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Tonor</t>
+          <t>Audio Array</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -5209,10 +5209,10 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>6523.73</v>
+        <v>5416.58</v>
       </c>
       <c r="F134" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G134" t="n">
         <v>0</v>
@@ -5221,16 +5221,16 @@
         <v>0</v>
       </c>
       <c r="I134" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J134" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>B0GW96SHSK</t>
+          <t>B0BPMBMN3S</t>
         </is>
       </c>
       <c r="B135" t="inlineStr"/>
@@ -5245,10 +5245,10 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>5761.02</v>
+        <v>5197.46</v>
       </c>
       <c r="F135" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G135" t="n">
         <v>0</v>
@@ -5257,22 +5257,22 @@
         <v>0</v>
       </c>
       <c r="I135" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J135" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>B0FN7FYZM3</t>
+          <t>B0BRCR2QQ7</t>
         </is>
       </c>
       <c r="B136" t="inlineStr"/>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Audio Array</t>
+          <t>Tonor</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -5281,10 +5281,10 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>5416.58</v>
+        <v>4744.07</v>
       </c>
       <c r="F136" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G136" t="n">
         <v>0</v>
@@ -5296,13 +5296,13 @@
         <v>1</v>
       </c>
       <c r="J136" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>B0BPMBMN3S</t>
+          <t>B0GW8Z556N</t>
         </is>
       </c>
       <c r="B137" t="inlineStr"/>
@@ -5317,10 +5317,10 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>5197.46</v>
+        <v>3903.64</v>
       </c>
       <c r="F137" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G137" t="n">
         <v>0</v>
@@ -5329,22 +5329,22 @@
         <v>0</v>
       </c>
       <c r="I137" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J137" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>B0DFMQCGT1</t>
+          <t>B09Z5Q194D</t>
         </is>
       </c>
       <c r="B138" t="inlineStr"/>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Audio Array</t>
+          <t>Tonor</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -5353,10 +5353,10 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>5019.5</v>
+        <v>3219.49</v>
       </c>
       <c r="F138" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G138" t="n">
         <v>0</v>
@@ -5365,22 +5365,22 @@
         <v>0</v>
       </c>
       <c r="I138" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J138" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>B0GW8Z556N</t>
+          <t>B0CFKZ72N7</t>
         </is>
       </c>
       <c r="B139" t="inlineStr"/>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Audio Array</t>
+          <t>Tonor</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -5389,10 +5389,10 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>3903.64</v>
+        <v>3007.63</v>
       </c>
       <c r="F139" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G139" t="n">
         <v>0</v>
@@ -5401,22 +5401,22 @@
         <v>0</v>
       </c>
       <c r="I139" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J139" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>B0CFKZ72N7</t>
+          <t>B0GW8R2RYM</t>
         </is>
       </c>
       <c r="B140" t="inlineStr"/>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Tonor</t>
+          <t>Audio Array</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -5425,10 +5425,10 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>3007.63</v>
+        <v>2710.16</v>
       </c>
       <c r="F140" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G140" t="n">
         <v>0</v>
@@ -5437,7 +5437,7 @@
         <v>0</v>
       </c>
       <c r="I140" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J140" t="n">
         <v>0</v>
@@ -5446,7 +5446,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>B0GW8R2RYM</t>
+          <t>B0DFMQCGT1</t>
         </is>
       </c>
       <c r="B141" t="inlineStr"/>
@@ -5461,10 +5461,10 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>2710.16</v>
+        <v>2477.97</v>
       </c>
       <c r="F141" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G141" t="n">
         <v>0</v>
@@ -5473,7 +5473,7 @@
         <v>0</v>
       </c>
       <c r="I141" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J141" t="n">
         <v>0</v>
@@ -5482,13 +5482,13 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>B0BRCR2QQ7</t>
+          <t>B0C4YT43Z3</t>
         </is>
       </c>
       <c r="B142" t="inlineStr"/>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Tonor</t>
+          <t>Audio Array</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -5497,7 +5497,7 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>2372.04</v>
+        <v>1863.56</v>
       </c>
       <c r="F142" t="n">
         <v>1</v>
@@ -5512,13 +5512,13 @@
         <v>1</v>
       </c>
       <c r="J142" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>B0C4YT43Z3</t>
+          <t>B0B4G5ZLTB</t>
         </is>
       </c>
       <c r="B143" t="inlineStr"/>

</xml_diff>